<commit_message>
Diseño del informe Excel más fiel al PDF
- Encabezado institucional en una sola línea (combinado C:G, alturas
  por línea) — en la vista de Excel el texto se encimaba
- Ficha técnica compacta y pareja (filas de 20px)
- Código de ensayo más visible (11pt blanco)
- Botón ACTUALIZAR REPORTE reubicado sobre la franja de código
  (antes pisaba el encabezado)
</commit_message>
<xml_diff>
--- a/backend/templates/base/base_granulometria.xlsx
+++ b/backend/templates/base/base_granulometria.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot; %&quot;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,7 +74,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -102,6 +102,12 @@
     <font>
       <name val="Calibri"/>
       <color rgb="001D4ED8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -229,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -295,6 +301,9 @@
     <xf numFmtId="164" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -306,11 +315,11 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -871,7 +880,7 @@
     <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>GOBIERNO REGIONAL CUSCO</t>
@@ -885,28 +894,28 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3" ht="12" customHeight="1">
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>SUB GERENCIA DE COBERTURA Y COMUNICACIONES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="12" customHeight="1">
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>UNIDAD FUNCIONAL ESTUDIOS Y PROYECTOS</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="14" customHeight="1">
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Laboratorio de Mecánica de Suelos, Materiales y Pavimentos</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="12" customHeight="1">
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>«Año de la recuperación y consolidación de la economía peruana»</t>
@@ -930,7 +939,7 @@
       <c r="I8" s="7" t="n"/>
     </row>
     <row r="9" ht="6" customHeight="1"/>
-    <row r="10">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>PROYECTO</t>
@@ -945,7 +954,7 @@
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>UBICACIÓN</t>
@@ -976,7 +985,7 @@
       </c>
       <c r="I11" s="10" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>SOLICITANTE</t>
@@ -993,7 +1002,7 @@
       <c r="F12" s="14" t="n"/>
       <c r="G12" s="15" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>COORDENADAS</t>
@@ -1018,7 +1027,7 @@
       </c>
       <c r="I13" s="10" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>DATOS DE MUESTRA</t>
@@ -1177,32 +1186,32 @@
       <c r="I23" s="17" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Tamiz</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Masa (g)</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>% Ret Parcial</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>% Ret Acum.</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="23" t="inlineStr">
         <is>
           <t>% que Pasa</t>
         </is>
@@ -1217,19 +1226,19 @@
           <t>3"</t>
         </is>
       </c>
-      <c r="B25" s="23" t="n">
+      <c r="B25" s="24" t="n">
         <v>75</v>
       </c>
       <c r="C25" s="19" t="n"/>
-      <c r="D25" s="24">
+      <c r="D25" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C25)),IFERROR(C25/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="25">
         <f>IF(ISNUMBER(D25),D25,0)</f>
         <v/>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="25">
         <f>100-E25</f>
         <v/>
       </c>
@@ -1243,19 +1252,19 @@
           <t>2 1/2"</t>
         </is>
       </c>
-      <c r="B26" s="23" t="n">
+      <c r="B26" s="24" t="n">
         <v>62.9</v>
       </c>
       <c r="C26" s="19" t="n"/>
-      <c r="D26" s="24">
+      <c r="D26" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C26)),IFERROR(C26/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E26" s="24">
+      <c r="E26" s="25">
         <f>IF(ISNUMBER(D26),E25+D26,E25)</f>
         <v/>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="25">
         <f>100-E26</f>
         <v/>
       </c>
@@ -1269,19 +1278,19 @@
           <t>2"</t>
         </is>
       </c>
-      <c r="B27" s="23" t="n">
+      <c r="B27" s="24" t="n">
         <v>50.8</v>
       </c>
       <c r="C27" s="19" t="n"/>
-      <c r="D27" s="24">
+      <c r="D27" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C27)),IFERROR(C27/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E27" s="24">
+      <c r="E27" s="25">
         <f>IF(ISNUMBER(D27),E26+D27,E26)</f>
         <v/>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="25">
         <f>100-E27</f>
         <v/>
       </c>
@@ -1295,19 +1304,19 @@
           <t>1 1/2"</t>
         </is>
       </c>
-      <c r="B28" s="23" t="n">
+      <c r="B28" s="24" t="n">
         <v>38.1</v>
       </c>
       <c r="C28" s="19" t="n"/>
-      <c r="D28" s="24">
+      <c r="D28" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C28)),IFERROR(C28/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E28" s="24">
+      <c r="E28" s="25">
         <f>IF(ISNUMBER(D28),E27+D28,E27)</f>
         <v/>
       </c>
-      <c r="F28" s="24">
+      <c r="F28" s="25">
         <f>100-E28</f>
         <v/>
       </c>
@@ -1321,19 +1330,19 @@
           <t>1"</t>
         </is>
       </c>
-      <c r="B29" s="23" t="n">
+      <c r="B29" s="24" t="n">
         <v>25.4</v>
       </c>
       <c r="C29" s="19" t="n"/>
-      <c r="D29" s="24">
+      <c r="D29" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C29)),IFERROR(C29/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E29" s="24">
+      <c r="E29" s="25">
         <f>IF(ISNUMBER(D29),E28+D29,E28)</f>
         <v/>
       </c>
-      <c r="F29" s="24">
+      <c r="F29" s="25">
         <f>100-E29</f>
         <v/>
       </c>
@@ -1347,19 +1356,19 @@
           <t>3/4"</t>
         </is>
       </c>
-      <c r="B30" s="23" t="n">
+      <c r="B30" s="24" t="n">
         <v>19</v>
       </c>
       <c r="C30" s="19" t="n"/>
-      <c r="D30" s="24">
+      <c r="D30" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C30)),IFERROR(C30/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E30" s="24">
+      <c r="E30" s="25">
         <f>IF(ISNUMBER(D30),E29+D30,E29)</f>
         <v/>
       </c>
-      <c r="F30" s="24">
+      <c r="F30" s="25">
         <f>100-E30</f>
         <v/>
       </c>
@@ -1373,19 +1382,19 @@
           <t>1/2"</t>
         </is>
       </c>
-      <c r="B31" s="23" t="n">
+      <c r="B31" s="24" t="n">
         <v>12.7</v>
       </c>
       <c r="C31" s="19" t="n"/>
-      <c r="D31" s="24">
+      <c r="D31" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C31)),IFERROR(C31/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E31" s="24">
+      <c r="E31" s="25">
         <f>IF(ISNUMBER(D31),E30+D31,E30)</f>
         <v/>
       </c>
-      <c r="F31" s="24">
+      <c r="F31" s="25">
         <f>100-E31</f>
         <v/>
       </c>
@@ -1399,19 +1408,19 @@
           <t>3/8"</t>
         </is>
       </c>
-      <c r="B32" s="23" t="n">
+      <c r="B32" s="24" t="n">
         <v>9.5</v>
       </c>
       <c r="C32" s="19" t="n"/>
-      <c r="D32" s="24">
+      <c r="D32" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C32)),IFERROR(C32/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E32" s="24">
+      <c r="E32" s="25">
         <f>IF(ISNUMBER(D32),E31+D32,E31)</f>
         <v/>
       </c>
-      <c r="F32" s="24">
+      <c r="F32" s="25">
         <f>100-E32</f>
         <v/>
       </c>
@@ -1425,19 +1434,19 @@
           <t>1/4"</t>
         </is>
       </c>
-      <c r="B33" s="23" t="n">
+      <c r="B33" s="24" t="n">
         <v>6.3</v>
       </c>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="24">
+      <c r="D33" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C33)),IFERROR(C33/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E33" s="24">
+      <c r="E33" s="25">
         <f>IF(ISNUMBER(D33),E32+D33,E32)</f>
         <v/>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="25">
         <f>100-E33</f>
         <v/>
       </c>
@@ -1451,19 +1460,19 @@
           <t>N° 4</t>
         </is>
       </c>
-      <c r="B34" s="23" t="n">
+      <c r="B34" s="24" t="n">
         <v>4.76</v>
       </c>
       <c r="C34" s="19" t="n"/>
-      <c r="D34" s="24">
+      <c r="D34" s="25">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C34)),IFERROR(C34/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E34" s="24">
+      <c r="E34" s="25">
         <f>IF(ISNUMBER(D34),E33+D34,E33)</f>
         <v/>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="25">
         <f>100-E34</f>
         <v/>
       </c>
@@ -1477,19 +1486,19 @@
           <t>N° 8</t>
         </is>
       </c>
-      <c r="B35" s="23" t="n">
+      <c r="B35" s="24" t="n">
         <v>2.36</v>
       </c>
       <c r="C35" s="19" t="n"/>
-      <c r="D35" s="24">
+      <c r="D35" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C35)),IFERROR(C35/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E35" s="24">
+      <c r="E35" s="25">
         <f>IF(ISNUMBER(D35),E34+D35,E34)</f>
         <v/>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="25">
         <f>100-E35</f>
         <v/>
       </c>
@@ -1503,19 +1512,19 @@
           <t>N° 10</t>
         </is>
       </c>
-      <c r="B36" s="23" t="n">
+      <c r="B36" s="24" t="n">
         <v>2</v>
       </c>
       <c r="C36" s="19" t="n"/>
-      <c r="D36" s="24">
+      <c r="D36" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C36)),IFERROR(C36/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E36" s="24">
+      <c r="E36" s="25">
         <f>IF(ISNUMBER(D36),E35+D36,E35)</f>
         <v/>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="25">
         <f>100-E36</f>
         <v/>
       </c>
@@ -1529,19 +1538,19 @@
           <t>N° 16</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n">
+      <c r="B37" s="24" t="n">
         <v>1.1</v>
       </c>
       <c r="C37" s="19" t="n"/>
-      <c r="D37" s="24">
+      <c r="D37" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C37)),IFERROR(C37/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="25">
         <f>IF(ISNUMBER(D37),E36+D37,E36)</f>
         <v/>
       </c>
-      <c r="F37" s="24">
+      <c r="F37" s="25">
         <f>100-E37</f>
         <v/>
       </c>
@@ -1555,19 +1564,19 @@
           <t>N° 20</t>
         </is>
       </c>
-      <c r="B38" s="23" t="n">
+      <c r="B38" s="24" t="n">
         <v>0.85</v>
       </c>
       <c r="C38" s="19" t="n"/>
-      <c r="D38" s="24">
+      <c r="D38" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C38)),IFERROR(C38/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E38" s="24">
+      <c r="E38" s="25">
         <f>IF(ISNUMBER(D38),E37+D38,E37)</f>
         <v/>
       </c>
-      <c r="F38" s="24">
+      <c r="F38" s="25">
         <f>100-E38</f>
         <v/>
       </c>
@@ -1581,19 +1590,19 @@
           <t>N° 30</t>
         </is>
       </c>
-      <c r="B39" s="23" t="n">
+      <c r="B39" s="24" t="n">
         <v>0.59</v>
       </c>
       <c r="C39" s="19" t="n"/>
-      <c r="D39" s="24">
+      <c r="D39" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C39)),IFERROR(C39/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E39" s="24">
+      <c r="E39" s="25">
         <f>IF(ISNUMBER(D39),E38+D39,E38)</f>
         <v/>
       </c>
-      <c r="F39" s="24">
+      <c r="F39" s="25">
         <f>100-E39</f>
         <v/>
       </c>
@@ -1607,19 +1616,19 @@
           <t>N° 40</t>
         </is>
       </c>
-      <c r="B40" s="23" t="n">
+      <c r="B40" s="24" t="n">
         <v>0.425</v>
       </c>
       <c r="C40" s="19" t="n"/>
-      <c r="D40" s="24">
+      <c r="D40" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C40)),IFERROR(C40/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E40" s="24">
+      <c r="E40" s="25">
         <f>IF(ISNUMBER(D40),E39+D40,E39)</f>
         <v/>
       </c>
-      <c r="F40" s="24">
+      <c r="F40" s="25">
         <f>100-E40</f>
         <v/>
       </c>
@@ -1633,19 +1642,19 @@
           <t>N° 50</t>
         </is>
       </c>
-      <c r="B41" s="23" t="n">
+      <c r="B41" s="24" t="n">
         <v>0.297</v>
       </c>
       <c r="C41" s="19" t="n"/>
-      <c r="D41" s="24">
+      <c r="D41" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C41)),IFERROR(C41/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="25">
         <f>IF(ISNUMBER(D41),E40+D41,E40)</f>
         <v/>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="25">
         <f>100-E41</f>
         <v/>
       </c>
@@ -1659,19 +1668,19 @@
           <t>N° 60</t>
         </is>
       </c>
-      <c r="B42" s="23" t="n">
+      <c r="B42" s="24" t="n">
         <v>0.25</v>
       </c>
       <c r="C42" s="19" t="n"/>
-      <c r="D42" s="24">
+      <c r="D42" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C42)),IFERROR(C42/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E42" s="24">
+      <c r="E42" s="25">
         <f>IF(ISNUMBER(D42),E41+D42,E41)</f>
         <v/>
       </c>
-      <c r="F42" s="24">
+      <c r="F42" s="25">
         <f>100-E42</f>
         <v/>
       </c>
@@ -1685,19 +1694,19 @@
           <t>N° 100</t>
         </is>
       </c>
-      <c r="B43" s="23" t="n">
+      <c r="B43" s="24" t="n">
         <v>0.149</v>
       </c>
       <c r="C43" s="19" t="n"/>
-      <c r="D43" s="24">
+      <c r="D43" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C43)),IFERROR(C43/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E43" s="24">
+      <c r="E43" s="25">
         <f>IF(ISNUMBER(D43),E42+D43,E42)</f>
         <v/>
       </c>
-      <c r="F43" s="24">
+      <c r="F43" s="25">
         <f>100-E43</f>
         <v/>
       </c>
@@ -1711,19 +1720,19 @@
           <t>N° 140</t>
         </is>
       </c>
-      <c r="B44" s="23" t="n">
+      <c r="B44" s="24" t="n">
         <v>0.106</v>
       </c>
       <c r="C44" s="19" t="n"/>
-      <c r="D44" s="24">
+      <c r="D44" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C44)),IFERROR(C44/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E44" s="24">
+      <c r="E44" s="25">
         <f>IF(ISNUMBER(D44),E43+D44,E43)</f>
         <v/>
       </c>
-      <c r="F44" s="24">
+      <c r="F44" s="25">
         <f>100-E44</f>
         <v/>
       </c>
@@ -1737,19 +1746,19 @@
           <t>N° 200</t>
         </is>
       </c>
-      <c r="B45" s="23" t="n">
+      <c r="B45" s="24" t="n">
         <v>0.075</v>
       </c>
       <c r="C45" s="19" t="n"/>
-      <c r="D45" s="24">
+      <c r="D45" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C45)),IFERROR(C45/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E45" s="24">
+      <c r="E45" s="25">
         <f>IF(ISNUMBER(D45),E44+D45,E44)</f>
         <v/>
       </c>
-      <c r="F45" s="24">
+      <c r="F45" s="25">
         <f>100-E45</f>
         <v/>
       </c>
@@ -1764,19 +1773,19 @@
         </is>
       </c>
       <c r="B46" s="19" t="n"/>
-      <c r="C46" s="25">
+      <c r="C46" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0),MAX(F17-SUM(C35:C45),0),"")</f>
         <v/>
       </c>
-      <c r="D46" s="24">
+      <c r="D46" s="25">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C46)),IFERROR(C46/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E46" s="24">
+      <c r="E46" s="25">
         <f>IF(ISNUMBER(D46),E45+D46,E45)</f>
         <v/>
       </c>
-      <c r="F46" s="24">
+      <c r="F46" s="25">
         <f>100-E46</f>
         <v/>
       </c>
@@ -1788,19 +1797,19 @@
         </is>
       </c>
       <c r="B47" s="19" t="n"/>
-      <c r="C47" s="25">
+      <c r="C47" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C25)),SUM(C25:C34)+N(F17),"")</f>
         <v/>
       </c>
-      <c r="D47" s="24">
+      <c r="D47" s="25">
         <f>IF(ISNUMBER(C47),100,"")</f>
         <v/>
       </c>
-      <c r="E47" s="24">
+      <c r="E47" s="25">
         <f>IF(ISNUMBER(D47),SUM(D25:D46),"")</f>
         <v/>
       </c>
-      <c r="F47" s="24">
+      <c r="F47" s="25">
         <f>IF(ISNUMBER(E47),100-E47,"")</f>
         <v/>
       </c>
@@ -1826,7 +1835,7 @@
           <t>% GRAVA</t>
         </is>
       </c>
-      <c r="B50" s="26">
+      <c r="B50" s="27">
         <f>IF(ISNUMBER(E34),E34,"")</f>
         <v/>
       </c>
@@ -1835,7 +1844,7 @@
           <t>% ARENA</t>
         </is>
       </c>
-      <c r="D50" s="26">
+      <c r="D50" s="27">
         <f>IF(AND(ISNUMBER(F34),ISNUMBER(F45)),F34-F45,"")</f>
         <v/>
       </c>
@@ -1845,7 +1854,7 @@
           <t>% FINOS</t>
         </is>
       </c>
-      <c r="G50" s="26">
+      <c r="G50" s="27">
         <f>IF(ISNUMBER(F45),F45,"")</f>
         <v/>
       </c>
@@ -1858,7 +1867,7 @@
           <t>TMN</t>
         </is>
       </c>
-      <c r="B51" s="27">
+      <c r="B51" s="28">
         <f>IFERROR(INDEX(A25:A45,MATCH(TRUE,INDEX(E25:E45&gt;0.01,0),0)),"N/A")</f>
         <v/>
       </c>
@@ -1880,13 +1889,13 @@
       <c r="I53" s="17" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>SUCS</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="23" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
@@ -1905,7 +1914,7 @@
         </is>
       </c>
       <c r="B55" s="19" t="n"/>
-      <c r="C55" s="28" t="inlineStr">
+      <c r="C55" s="29" t="inlineStr">
         <is>
           <t>Gravas bien graduadas, mezclas grava-arena, pocos finos o sin finos.</t>
         </is>
@@ -1924,7 +1933,7 @@
         </is>
       </c>
       <c r="B56" s="19" t="n"/>
-      <c r="C56" s="28" t="inlineStr">
+      <c r="C56" s="29" t="inlineStr">
         <is>
           <t>Gravas mal graduadas, mezclas grava-arena, pocos finos o sin finos.</t>
         </is>
@@ -1943,7 +1952,7 @@
         </is>
       </c>
       <c r="B57" s="19" t="n"/>
-      <c r="C57" s="28" t="inlineStr">
+      <c r="C57" s="29" t="inlineStr">
         <is>
           <t>Gravas limosas, mezclas grava-arena-limo.</t>
         </is>
@@ -1962,7 +1971,7 @@
         </is>
       </c>
       <c r="B58" s="19" t="n"/>
-      <c r="C58" s="28" t="inlineStr">
+      <c r="C58" s="29" t="inlineStr">
         <is>
           <t>Gravas arcillosas, mezclas grava-arena-arcilla.</t>
         </is>
@@ -1981,7 +1990,7 @@
         </is>
       </c>
       <c r="B59" s="19" t="n"/>
-      <c r="C59" s="28" t="inlineStr">
+      <c r="C59" s="29" t="inlineStr">
         <is>
           <t>Arenas bien graduadas, arenas con grava, pocos finos o sin finos.</t>
         </is>
@@ -2000,7 +2009,7 @@
         </is>
       </c>
       <c r="B60" s="19" t="n"/>
-      <c r="C60" s="28" t="inlineStr">
+      <c r="C60" s="29" t="inlineStr">
         <is>
           <t>Arenas mal graduadas, arenas con grava, pocos finos o sin finos.</t>
         </is>
@@ -2019,7 +2028,7 @@
         </is>
       </c>
       <c r="B61" s="19" t="n"/>
-      <c r="C61" s="28" t="inlineStr">
+      <c r="C61" s="29" t="inlineStr">
         <is>
           <t>Arenas limosas, mezclas de arena y limo.</t>
         </is>
@@ -2038,7 +2047,7 @@
         </is>
       </c>
       <c r="B62" s="19" t="n"/>
-      <c r="C62" s="28" t="inlineStr">
+      <c r="C62" s="29" t="inlineStr">
         <is>
           <t>Arenas arcillosas, mezclas de arena y arcilla.</t>
         </is>
@@ -2057,7 +2066,7 @@
         </is>
       </c>
       <c r="B63" s="19" t="n"/>
-      <c r="C63" s="28" t="inlineStr">
+      <c r="C63" s="29" t="inlineStr">
         <is>
           <t>Limos inorgánicos y arenas muy finas, limos limpios, arenas finas, limosas o arcillosas.</t>
         </is>
@@ -2076,7 +2085,7 @@
         </is>
       </c>
       <c r="B64" s="19" t="n"/>
-      <c r="C64" s="28" t="inlineStr">
+      <c r="C64" s="29" t="inlineStr">
         <is>
           <t>Arcillas inorgánicas de plasticidad baja a media, arcillas con grava, arcillas arenosas.</t>
         </is>
@@ -2095,7 +2104,7 @@
         </is>
       </c>
       <c r="B65" s="19" t="n"/>
-      <c r="C65" s="28" t="inlineStr">
+      <c r="C65" s="29" t="inlineStr">
         <is>
           <t>Limos orgánicos y arcillas orgánicas limosas de baja plasticidad.</t>
         </is>
@@ -2114,7 +2123,7 @@
         </is>
       </c>
       <c r="B66" s="19" t="n"/>
-      <c r="C66" s="28" t="inlineStr">
+      <c r="C66" s="29" t="inlineStr">
         <is>
           <t>Limos inorgánicos, suelos arenosos finos o limosos con mica o diatomeas.</t>
         </is>
@@ -2133,7 +2142,7 @@
         </is>
       </c>
       <c r="B67" s="19" t="n"/>
-      <c r="C67" s="28" t="inlineStr">
+      <c r="C67" s="29" t="inlineStr">
         <is>
           <t>Arcillas inorgánicas de plasticidad alta.</t>
         </is>
@@ -2152,7 +2161,7 @@
         </is>
       </c>
       <c r="B68" s="19" t="n"/>
-      <c r="C68" s="28" t="inlineStr">
+      <c r="C68" s="29" t="inlineStr">
         <is>
           <t>Arcillas orgánicas de plasticidad media a alta.</t>
         </is>
@@ -2180,28 +2189,28 @@
       <c r="I70" s="17" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="29" t="n"/>
-      <c r="B101" s="29" t="n"/>
-      <c r="C101" s="29" t="n"/>
-      <c r="D101" s="29" t="n"/>
-      <c r="E101" s="29" t="n"/>
-      <c r="F101" s="29" t="n"/>
-      <c r="G101" s="29" t="n"/>
-      <c r="H101" s="29" t="n"/>
-      <c r="I101" s="29" t="n"/>
+      <c r="A101" s="30" t="n"/>
+      <c r="B101" s="30" t="n"/>
+      <c r="C101" s="30" t="n"/>
+      <c r="D101" s="30" t="n"/>
+      <c r="E101" s="30" t="n"/>
+      <c r="F101" s="30" t="n"/>
+      <c r="G101" s="30" t="n"/>
+      <c r="H101" s="30" t="n"/>
+      <c r="I101" s="30" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="30" t="inlineStr">
+      <c r="A102" s="31" t="inlineStr">
         <is>
           <t>ESP. ENSAYOS GEOTECNICOS</t>
         </is>
       </c>
-      <c r="D102" s="30" t="inlineStr">
+      <c r="D102" s="31" t="inlineStr">
         <is>
           <t>ESP. SUELOS Y PAVIMENTOS</t>
         </is>
       </c>
-      <c r="G102" s="30" t="inlineStr">
+      <c r="G102" s="31" t="inlineStr">
         <is>
           <t>SUPERVISOR</t>
         </is>
@@ -2215,47 +2224,47 @@
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="A59:B59"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="D19:E19"/>
     <mergeCell ref="A60:B60"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="A67:B67"/>
     <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C3:G3"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="D50:E50"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
+    <mergeCell ref="C4:G4"/>
     <mergeCell ref="B21:I21"/>
-    <mergeCell ref="C3:F3"/>
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="A65:B65"/>
     <mergeCell ref="D102:F102"/>
+    <mergeCell ref="C1:G1"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="F18:G18"/>
-    <mergeCell ref="C6:F6"/>
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A66:B66"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="A53:I53"/>
-    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="F17:G17"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="G50:I50"/>
     <mergeCell ref="A102:C102"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="C64:I64"/>
+    <mergeCell ref="C2:G2"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="C64:I64"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="F24:I24"/>
     <mergeCell ref="G102:I102"/>
-    <mergeCell ref="C1:F1"/>
     <mergeCell ref="G12:I12"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="D18:E18"/>
@@ -2275,7 +2284,7 @@
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="B12:D12"/>
-    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="A67:B67"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>

</xml_diff>

<commit_message>
Macro: botón ACTUALIZAR REPORTE al costado derecho del reporte
Quedaba encima del código centrado en la franja; ahora flota fuera
del área del informe (columna J, al costado de la franja CÓDIGO).
</commit_message>
<xml_diff>
--- a/backend/templates/base/base_granulometria.xlsx
+++ b/backend/templates/base/base_granulometria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Reporte" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="_DATOS" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="_GRAFICOS" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="_MAPA" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DATOS" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_GRAFICOS" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_MAPA" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="GranX">'_DATOS'!$A$3:$A$23</definedName>
@@ -399,13 +399,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -426,7 +426,7 @@
             <v>Curva Granulométrica</v>
           </tx>
           <spPr>
-            <a:ln w="24000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="24000">
               <a:solidFill>
                 <a:srgbClr val="1E40AF"/>
               </a:solidFill>
@@ -437,10 +437,10 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1E40AF"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -501,7 +501,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -516,9 +516,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -538,13 +538,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -563,13 +563,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>

<commit_message>
Ficha técnica pareja en los 3 informes Excel
Los valores de Ubicación y Coordenadas pasan a 9pt para que textos
como 'La Convención' y '0.00 - 0.20 m' no salten de línea y descuadren
las filas de la ficha (ahora todas a 20px, como el grid del PDF).
</commit_message>
<xml_diff>
--- a/backend/templates/base/base_granulometria.xlsx
+++ b/backend/templates/base/base_granulometria.xlsx
@@ -235,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -264,7 +264,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -280,6 +280,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1038,41 +1041,41 @@
           <t>Explor.:</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n"/>
+      <c r="C14" s="16" t="n"/>
       <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Progresiva:</t>
         </is>
       </c>
-      <c r="E14" s="10" t="n"/>
+      <c r="E14" s="16" t="n"/>
       <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Estrato:</t>
         </is>
       </c>
-      <c r="G14" s="10" t="n"/>
+      <c r="G14" s="16" t="n"/>
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Lado:</t>
         </is>
       </c>
-      <c r="I14" s="10" t="n"/>
+      <c r="I14" s="16" t="n"/>
     </row>
     <row r="15" ht="6" customHeight="1"/>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>ANÁLISIS GRANULOMÉTRICO POR TAMIZADO - MTC E 107</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="17" t="n"/>
-      <c r="I16" s="17" t="n"/>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="18" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -1080,16 +1083,16 @@
           <t>PESO TOTAL (g)</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="19" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="20" t="n"/>
       <c r="D17" s="13" t="inlineStr">
         <is>
           <t>PESO FRAC. FINA TAMIZADA (g)</t>
         </is>
       </c>
       <c r="E17" s="14" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -1097,22 +1100,22 @@
           <t>PESO FRACCIÓN GRUESA (g)</t>
         </is>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="21">
         <f>IF(N(B17)&gt;0,SUM(C25:C34),"")</f>
         <v/>
       </c>
-      <c r="C18" s="21" t="n"/>
+      <c r="C18" s="22" t="n"/>
       <c r="D18" s="13" t="inlineStr">
         <is>
           <t>PESO MUESTRA LAVADA (g)</t>
         </is>
       </c>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="20">
+      <c r="F18" s="21">
         <f>IF(AND(N(B17)&gt;0,N(F17)&gt;0),B18+SUM(C35:C45)*B19/F17,"")</f>
         <v/>
       </c>
-      <c r="G18" s="21" t="n"/>
+      <c r="G18" s="22" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -1120,22 +1123,22 @@
           <t>PESO FRACCIÓN FINA (g)</t>
         </is>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="21">
         <f>IF(N(B17)&gt;0,B17-B18,"")</f>
         <v/>
       </c>
-      <c r="C19" s="21" t="n"/>
+      <c r="C19" s="22" t="n"/>
       <c r="D19" s="13" t="inlineStr">
         <is>
           <t>COEFICIENTE</t>
         </is>
       </c>
       <c r="E19" s="14" t="n"/>
-      <c r="F19" s="22">
+      <c r="F19" s="23">
         <f>IF(AND(N(B17)&gt;0,N(F17)&gt;0),IFERROR(F17/B17,0),"")</f>
         <v/>
       </c>
-      <c r="G19" s="21" t="n"/>
+      <c r="G19" s="22" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -1143,16 +1146,16 @@
           <t>LÍMITE LÍQUIDO (%)</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="19" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="20" t="n"/>
       <c r="D20" s="13" t="inlineStr">
         <is>
           <t>ÍNDICE DE PLASTICIDAD (%)</t>
         </is>
       </c>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -1160,58 +1163,58 @@
           <t>GRADACIÓN</t>
         </is>
       </c>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="19" t="n"/>
-      <c r="G21" s="19" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="20" t="n"/>
+      <c r="D21" s="20" t="n"/>
+      <c r="E21" s="20" t="n"/>
+      <c r="F21" s="20" t="n"/>
+      <c r="G21" s="20" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="20" t="n"/>
     </row>
     <row r="22" ht="6" customHeight="1"/>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>TAMIZADO</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
-      <c r="G23" s="17" t="n"/>
-      <c r="H23" s="17" t="n"/>
-      <c r="I23" s="17" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Tamiz</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Masa (g)</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="24" t="inlineStr">
         <is>
           <t>% Ret Parcial</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>% Ret Acum.</t>
         </is>
       </c>
-      <c r="F24" s="23" t="inlineStr">
+      <c r="F24" s="24" t="inlineStr">
         <is>
           <t>% que Pasa</t>
         </is>
@@ -1221,613 +1224,613 @@
       <c r="I24" s="7" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>3"</t>
         </is>
       </c>
-      <c r="B25" s="24" t="n">
+      <c r="B25" s="25" t="n">
         <v>75</v>
       </c>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="25">
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C25)),IFERROR(C25/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="26">
         <f>IF(ISNUMBER(D25),D25,0)</f>
         <v/>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="26">
         <f>100-E25</f>
         <v/>
       </c>
-      <c r="G25" s="19" t="n"/>
-      <c r="H25" s="19" t="n"/>
-      <c r="I25" s="19" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>2 1/2"</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n">
+      <c r="B26" s="25" t="n">
         <v>62.9</v>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="25">
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C26)),IFERROR(C26/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="26">
         <f>IF(ISNUMBER(D26),E25+D26,E25)</f>
         <v/>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="26">
         <f>100-E26</f>
         <v/>
       </c>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="19" t="n"/>
-      <c r="I26" s="19" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="20" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>2"</t>
         </is>
       </c>
-      <c r="B27" s="24" t="n">
+      <c r="B27" s="25" t="n">
         <v>50.8</v>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="25">
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C27)),IFERROR(C27/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E27" s="25">
+      <c r="E27" s="26">
         <f>IF(ISNUMBER(D27),E26+D27,E26)</f>
         <v/>
       </c>
-      <c r="F27" s="25">
+      <c r="F27" s="26">
         <f>100-E27</f>
         <v/>
       </c>
-      <c r="G27" s="19" t="n"/>
-      <c r="H27" s="19" t="n"/>
-      <c r="I27" s="19" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>1 1/2"</t>
         </is>
       </c>
-      <c r="B28" s="24" t="n">
+      <c r="B28" s="25" t="n">
         <v>38.1</v>
       </c>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="25">
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C28)),IFERROR(C28/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E28" s="25">
+      <c r="E28" s="26">
         <f>IF(ISNUMBER(D28),E27+D28,E27)</f>
         <v/>
       </c>
-      <c r="F28" s="25">
+      <c r="F28" s="26">
         <f>100-E28</f>
         <v/>
       </c>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
-      <c r="I28" s="19" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="20" t="n"/>
+      <c r="I28" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>1"</t>
         </is>
       </c>
-      <c r="B29" s="24" t="n">
+      <c r="B29" s="25" t="n">
         <v>25.4</v>
       </c>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="25">
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C29)),IFERROR(C29/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E29" s="25">
+      <c r="E29" s="26">
         <f>IF(ISNUMBER(D29),E28+D29,E28)</f>
         <v/>
       </c>
-      <c r="F29" s="25">
+      <c r="F29" s="26">
         <f>100-E29</f>
         <v/>
       </c>
-      <c r="G29" s="19" t="n"/>
-      <c r="H29" s="19" t="n"/>
-      <c r="I29" s="19" t="n"/>
+      <c r="G29" s="20" t="n"/>
+      <c r="H29" s="20" t="n"/>
+      <c r="I29" s="20" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>3/4"</t>
         </is>
       </c>
-      <c r="B30" s="24" t="n">
+      <c r="B30" s="25" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="25">
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C30)),IFERROR(C30/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E30" s="25">
+      <c r="E30" s="26">
         <f>IF(ISNUMBER(D30),E29+D30,E29)</f>
         <v/>
       </c>
-      <c r="F30" s="25">
+      <c r="F30" s="26">
         <f>100-E30</f>
         <v/>
       </c>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="19" t="n"/>
+      <c r="G30" s="20" t="n"/>
+      <c r="H30" s="20" t="n"/>
+      <c r="I30" s="20" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>1/2"</t>
         </is>
       </c>
-      <c r="B31" s="24" t="n">
+      <c r="B31" s="25" t="n">
         <v>12.7</v>
       </c>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="25">
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C31)),IFERROR(C31/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E31" s="25">
+      <c r="E31" s="26">
         <f>IF(ISNUMBER(D31),E30+D31,E30)</f>
         <v/>
       </c>
-      <c r="F31" s="25">
+      <c r="F31" s="26">
         <f>100-E31</f>
         <v/>
       </c>
-      <c r="G31" s="19" t="n"/>
-      <c r="H31" s="19" t="n"/>
-      <c r="I31" s="19" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="20" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>3/8"</t>
         </is>
       </c>
-      <c r="B32" s="24" t="n">
+      <c r="B32" s="25" t="n">
         <v>9.5</v>
       </c>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="25">
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C32)),IFERROR(C32/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E32" s="25">
+      <c r="E32" s="26">
         <f>IF(ISNUMBER(D32),E31+D32,E31)</f>
         <v/>
       </c>
-      <c r="F32" s="25">
+      <c r="F32" s="26">
         <f>100-E32</f>
         <v/>
       </c>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="19" t="n"/>
+      <c r="G32" s="20" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>1/4"</t>
         </is>
       </c>
-      <c r="B33" s="24" t="n">
+      <c r="B33" s="25" t="n">
         <v>6.3</v>
       </c>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="25">
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C33)),IFERROR(C33/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E33" s="25">
+      <c r="E33" s="26">
         <f>IF(ISNUMBER(D33),E32+D33,E32)</f>
         <v/>
       </c>
-      <c r="F33" s="25">
+      <c r="F33" s="26">
         <f>100-E33</f>
         <v/>
       </c>
-      <c r="G33" s="19" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="19" t="n"/>
+      <c r="G33" s="20" t="n"/>
+      <c r="H33" s="20" t="n"/>
+      <c r="I33" s="20" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>N° 4</t>
         </is>
       </c>
-      <c r="B34" s="24" t="n">
+      <c r="B34" s="25" t="n">
         <v>4.76</v>
       </c>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="25">
+      <c r="C34" s="20" t="n"/>
+      <c r="D34" s="26">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C34)),IFERROR(C34/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="26">
         <f>IF(ISNUMBER(D34),E33+D34,E33)</f>
         <v/>
       </c>
-      <c r="F34" s="25">
+      <c r="F34" s="26">
         <f>100-E34</f>
         <v/>
       </c>
-      <c r="G34" s="19" t="n"/>
-      <c r="H34" s="19" t="n"/>
-      <c r="I34" s="19" t="n"/>
+      <c r="G34" s="20" t="n"/>
+      <c r="H34" s="20" t="n"/>
+      <c r="I34" s="20" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>N° 8</t>
         </is>
       </c>
-      <c r="B35" s="24" t="n">
+      <c r="B35" s="25" t="n">
         <v>2.36</v>
       </c>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="25">
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C35)),IFERROR(C35/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E35" s="25">
+      <c r="E35" s="26">
         <f>IF(ISNUMBER(D35),E34+D35,E34)</f>
         <v/>
       </c>
-      <c r="F35" s="25">
+      <c r="F35" s="26">
         <f>100-E35</f>
         <v/>
       </c>
-      <c r="G35" s="19" t="n"/>
-      <c r="H35" s="19" t="n"/>
-      <c r="I35" s="19" t="n"/>
+      <c r="G35" s="20" t="n"/>
+      <c r="H35" s="20" t="n"/>
+      <c r="I35" s="20" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>N° 10</t>
         </is>
       </c>
-      <c r="B36" s="24" t="n">
+      <c r="B36" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="25">
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C36)),IFERROR(C36/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E36" s="25">
+      <c r="E36" s="26">
         <f>IF(ISNUMBER(D36),E35+D36,E35)</f>
         <v/>
       </c>
-      <c r="F36" s="25">
+      <c r="F36" s="26">
         <f>100-E36</f>
         <v/>
       </c>
-      <c r="G36" s="19" t="n"/>
-      <c r="H36" s="19" t="n"/>
-      <c r="I36" s="19" t="n"/>
+      <c r="G36" s="20" t="n"/>
+      <c r="H36" s="20" t="n"/>
+      <c r="I36" s="20" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>N° 16</t>
         </is>
       </c>
-      <c r="B37" s="24" t="n">
+      <c r="B37" s="25" t="n">
         <v>1.1</v>
       </c>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="25">
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C37)),IFERROR(C37/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E37" s="25">
+      <c r="E37" s="26">
         <f>IF(ISNUMBER(D37),E36+D37,E36)</f>
         <v/>
       </c>
-      <c r="F37" s="25">
+      <c r="F37" s="26">
         <f>100-E37</f>
         <v/>
       </c>
-      <c r="G37" s="19" t="n"/>
-      <c r="H37" s="19" t="n"/>
-      <c r="I37" s="19" t="n"/>
+      <c r="G37" s="20" t="n"/>
+      <c r="H37" s="20" t="n"/>
+      <c r="I37" s="20" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>N° 20</t>
         </is>
       </c>
-      <c r="B38" s="24" t="n">
+      <c r="B38" s="25" t="n">
         <v>0.85</v>
       </c>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="25">
+      <c r="C38" s="20" t="n"/>
+      <c r="D38" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C38)),IFERROR(C38/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="26">
         <f>IF(ISNUMBER(D38),E37+D38,E37)</f>
         <v/>
       </c>
-      <c r="F38" s="25">
+      <c r="F38" s="26">
         <f>100-E38</f>
         <v/>
       </c>
-      <c r="G38" s="19" t="n"/>
-      <c r="H38" s="19" t="n"/>
-      <c r="I38" s="19" t="n"/>
+      <c r="G38" s="20" t="n"/>
+      <c r="H38" s="20" t="n"/>
+      <c r="I38" s="20" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr">
         <is>
           <t>N° 30</t>
         </is>
       </c>
-      <c r="B39" s="24" t="n">
+      <c r="B39" s="25" t="n">
         <v>0.59</v>
       </c>
-      <c r="C39" s="19" t="n"/>
-      <c r="D39" s="25">
+      <c r="C39" s="20" t="n"/>
+      <c r="D39" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C39)),IFERROR(C39/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="26">
         <f>IF(ISNUMBER(D39),E38+D39,E38)</f>
         <v/>
       </c>
-      <c r="F39" s="25">
+      <c r="F39" s="26">
         <f>100-E39</f>
         <v/>
       </c>
-      <c r="G39" s="19" t="n"/>
-      <c r="H39" s="19" t="n"/>
-      <c r="I39" s="19" t="n"/>
+      <c r="G39" s="20" t="n"/>
+      <c r="H39" s="20" t="n"/>
+      <c r="I39" s="20" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" s="20" t="inlineStr">
         <is>
           <t>N° 40</t>
         </is>
       </c>
-      <c r="B40" s="24" t="n">
+      <c r="B40" s="25" t="n">
         <v>0.425</v>
       </c>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="25">
+      <c r="C40" s="20" t="n"/>
+      <c r="D40" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C40)),IFERROR(C40/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E40" s="25">
+      <c r="E40" s="26">
         <f>IF(ISNUMBER(D40),E39+D40,E39)</f>
         <v/>
       </c>
-      <c r="F40" s="25">
+      <c r="F40" s="26">
         <f>100-E40</f>
         <v/>
       </c>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
+      <c r="G40" s="20" t="n"/>
+      <c r="H40" s="20" t="n"/>
+      <c r="I40" s="20" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>N° 50</t>
         </is>
       </c>
-      <c r="B41" s="24" t="n">
+      <c r="B41" s="25" t="n">
         <v>0.297</v>
       </c>
-      <c r="C41" s="19" t="n"/>
-      <c r="D41" s="25">
+      <c r="C41" s="20" t="n"/>
+      <c r="D41" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C41)),IFERROR(C41/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E41" s="25">
+      <c r="E41" s="26">
         <f>IF(ISNUMBER(D41),E40+D41,E40)</f>
         <v/>
       </c>
-      <c r="F41" s="25">
+      <c r="F41" s="26">
         <f>100-E41</f>
         <v/>
       </c>
-      <c r="G41" s="19" t="n"/>
-      <c r="H41" s="19" t="n"/>
-      <c r="I41" s="19" t="n"/>
+      <c r="G41" s="20" t="n"/>
+      <c r="H41" s="20" t="n"/>
+      <c r="I41" s="20" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="inlineStr">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>N° 60</t>
         </is>
       </c>
-      <c r="B42" s="24" t="n">
+      <c r="B42" s="25" t="n">
         <v>0.25</v>
       </c>
-      <c r="C42" s="19" t="n"/>
-      <c r="D42" s="25">
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C42)),IFERROR(C42/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="26">
         <f>IF(ISNUMBER(D42),E41+D42,E41)</f>
         <v/>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="26">
         <f>100-E42</f>
         <v/>
       </c>
-      <c r="G42" s="19" t="n"/>
-      <c r="H42" s="19" t="n"/>
-      <c r="I42" s="19" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="n"/>
+      <c r="I42" s="20" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>N° 100</t>
         </is>
       </c>
-      <c r="B43" s="24" t="n">
+      <c r="B43" s="25" t="n">
         <v>0.149</v>
       </c>
-      <c r="C43" s="19" t="n"/>
-      <c r="D43" s="25">
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C43)),IFERROR(C43/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E43" s="25">
+      <c r="E43" s="26">
         <f>IF(ISNUMBER(D43),E42+D43,E42)</f>
         <v/>
       </c>
-      <c r="F43" s="25">
+      <c r="F43" s="26">
         <f>100-E43</f>
         <v/>
       </c>
-      <c r="G43" s="19" t="n"/>
-      <c r="H43" s="19" t="n"/>
-      <c r="I43" s="19" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>N° 140</t>
         </is>
       </c>
-      <c r="B44" s="24" t="n">
+      <c r="B44" s="25" t="n">
         <v>0.106</v>
       </c>
-      <c r="C44" s="19" t="n"/>
-      <c r="D44" s="25">
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C44)),IFERROR(C44/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E44" s="25">
+      <c r="E44" s="26">
         <f>IF(ISNUMBER(D44),E43+D44,E43)</f>
         <v/>
       </c>
-      <c r="F44" s="25">
+      <c r="F44" s="26">
         <f>100-E44</f>
         <v/>
       </c>
-      <c r="G44" s="19" t="n"/>
-      <c r="H44" s="19" t="n"/>
-      <c r="I44" s="19" t="n"/>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>N° 200</t>
         </is>
       </c>
-      <c r="B45" s="24" t="n">
+      <c r="B45" s="25" t="n">
         <v>0.075</v>
       </c>
-      <c r="C45" s="19" t="n"/>
-      <c r="D45" s="25">
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C45)),IFERROR(C45/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E45" s="25">
+      <c r="E45" s="26">
         <f>IF(ISNUMBER(D45),E44+D45,E44)</f>
         <v/>
       </c>
-      <c r="F45" s="25">
+      <c r="F45" s="26">
         <f>100-E45</f>
         <v/>
       </c>
-      <c r="G45" s="19" t="n"/>
-      <c r="H45" s="19" t="n"/>
-      <c r="I45" s="19" t="n"/>
+      <c r="G45" s="20" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>&lt; N° 200</t>
         </is>
       </c>
-      <c r="B46" s="19" t="n"/>
-      <c r="C46" s="26">
+      <c r="B46" s="20" t="n"/>
+      <c r="C46" s="27">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0),MAX(F17-SUM(C35:C45),0),"")</f>
         <v/>
       </c>
-      <c r="D46" s="25">
+      <c r="D46" s="26">
         <f>IF(AND(N(F17)&gt;0,N(B17)&gt;0,ISNUMBER(C46)),IFERROR(C46/F17*(B17-B18)/B17*100,0),"")</f>
         <v/>
       </c>
-      <c r="E46" s="25">
+      <c r="E46" s="26">
         <f>IF(ISNUMBER(D46),E45+D46,E45)</f>
         <v/>
       </c>
-      <c r="F46" s="25">
+      <c r="F46" s="26">
         <f>100-E46</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B47" s="19" t="n"/>
-      <c r="C47" s="26">
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="27">
         <f>IF(AND(N(B17)&gt;0,ISNUMBER(C25)),SUM(C25:C34)+N(F17),"")</f>
         <v/>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="26">
         <f>IF(ISNUMBER(C47),100,"")</f>
         <v/>
       </c>
-      <c r="E47" s="25">
+      <c r="E47" s="26">
         <f>IF(ISNUMBER(D47),SUM(D25:D46),"")</f>
         <v/>
       </c>
-      <c r="F47" s="25">
+      <c r="F47" s="26">
         <f>IF(ISNUMBER(E47),100-E47,"")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="17" t="n"/>
-      <c r="D49" s="17" t="n"/>
-      <c r="E49" s="17" t="n"/>
-      <c r="F49" s="17" t="n"/>
-      <c r="G49" s="17" t="n"/>
-      <c r="H49" s="17" t="n"/>
-      <c r="I49" s="17" t="n"/>
+      <c r="B49" s="18" t="n"/>
+      <c r="C49" s="18" t="n"/>
+      <c r="D49" s="18" t="n"/>
+      <c r="E49" s="18" t="n"/>
+      <c r="F49" s="18" t="n"/>
+      <c r="G49" s="18" t="n"/>
+      <c r="H49" s="18" t="n"/>
+      <c r="I49" s="18" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
@@ -1835,7 +1838,7 @@
           <t>% GRAVA</t>
         </is>
       </c>
-      <c r="B50" s="27">
+      <c r="B50" s="28">
         <f>IF(ISNUMBER(E34),E34,"")</f>
         <v/>
       </c>
@@ -1844,7 +1847,7 @@
           <t>% ARENA</t>
         </is>
       </c>
-      <c r="D50" s="27">
+      <c r="D50" s="28">
         <f>IF(AND(ISNUMBER(F34),ISNUMBER(F45)),F34-F45,"")</f>
         <v/>
       </c>
@@ -1854,7 +1857,7 @@
           <t>% FINOS</t>
         </is>
       </c>
-      <c r="G50" s="27">
+      <c r="G50" s="28">
         <f>IF(ISNUMBER(F45),F45,"")</f>
         <v/>
       </c>
@@ -1867,35 +1870,35 @@
           <t>TMN</t>
         </is>
       </c>
-      <c r="B51" s="28">
+      <c r="B51" s="29">
         <f>IFERROR(INDEX(A25:A45,MATCH(TRUE,INDEX(E25:E45&gt;0.01,0),0)),"N/A")</f>
         <v/>
       </c>
       <c r="C51" s="9" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN SUCS (REFERENCIA)</t>
         </is>
       </c>
-      <c r="B53" s="17" t="n"/>
-      <c r="C53" s="17" t="n"/>
-      <c r="D53" s="17" t="n"/>
-      <c r="E53" s="17" t="n"/>
-      <c r="F53" s="17" t="n"/>
-      <c r="G53" s="17" t="n"/>
-      <c r="H53" s="17" t="n"/>
-      <c r="I53" s="17" t="n"/>
+      <c r="B53" s="18" t="n"/>
+      <c r="C53" s="18" t="n"/>
+      <c r="D53" s="18" t="n"/>
+      <c r="E53" s="18" t="n"/>
+      <c r="F53" s="18" t="n"/>
+      <c r="G53" s="18" t="n"/>
+      <c r="H53" s="18" t="n"/>
+      <c r="I53" s="18" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="inlineStr">
+      <c r="A54" s="24" t="inlineStr">
         <is>
           <t>SUCS</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
-      <c r="C54" s="23" t="inlineStr">
+      <c r="C54" s="24" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
@@ -1908,309 +1911,309 @@
       <c r="I54" s="7" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="inlineStr">
+      <c r="A55" s="20" t="inlineStr">
         <is>
           <t>GW</t>
         </is>
       </c>
-      <c r="B55" s="19" t="n"/>
-      <c r="C55" s="29" t="inlineStr">
+      <c r="B55" s="20" t="n"/>
+      <c r="C55" s="30" t="inlineStr">
         <is>
           <t>Gravas bien graduadas, mezclas grava-arena, pocos finos o sin finos.</t>
         </is>
       </c>
-      <c r="D55" s="19" t="n"/>
-      <c r="E55" s="19" t="n"/>
-      <c r="F55" s="19" t="n"/>
-      <c r="G55" s="19" t="n"/>
-      <c r="H55" s="19" t="n"/>
-      <c r="I55" s="19" t="n"/>
+      <c r="D55" s="20" t="n"/>
+      <c r="E55" s="20" t="n"/>
+      <c r="F55" s="20" t="n"/>
+      <c r="G55" s="20" t="n"/>
+      <c r="H55" s="20" t="n"/>
+      <c r="I55" s="20" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="19" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
         <is>
           <t>GP</t>
         </is>
       </c>
-      <c r="B56" s="19" t="n"/>
-      <c r="C56" s="29" t="inlineStr">
+      <c r="B56" s="20" t="n"/>
+      <c r="C56" s="30" t="inlineStr">
         <is>
           <t>Gravas mal graduadas, mezclas grava-arena, pocos finos o sin finos.</t>
         </is>
       </c>
-      <c r="D56" s="19" t="n"/>
-      <c r="E56" s="19" t="n"/>
-      <c r="F56" s="19" t="n"/>
-      <c r="G56" s="19" t="n"/>
-      <c r="H56" s="19" t="n"/>
-      <c r="I56" s="19" t="n"/>
+      <c r="D56" s="20" t="n"/>
+      <c r="E56" s="20" t="n"/>
+      <c r="F56" s="20" t="n"/>
+      <c r="G56" s="20" t="n"/>
+      <c r="H56" s="20" t="n"/>
+      <c r="I56" s="20" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="A57" s="20" t="inlineStr">
         <is>
           <t>GM</t>
         </is>
       </c>
-      <c r="B57" s="19" t="n"/>
-      <c r="C57" s="29" t="inlineStr">
+      <c r="B57" s="20" t="n"/>
+      <c r="C57" s="30" t="inlineStr">
         <is>
           <t>Gravas limosas, mezclas grava-arena-limo.</t>
         </is>
       </c>
-      <c r="D57" s="19" t="n"/>
-      <c r="E57" s="19" t="n"/>
-      <c r="F57" s="19" t="n"/>
-      <c r="G57" s="19" t="n"/>
-      <c r="H57" s="19" t="n"/>
-      <c r="I57" s="19" t="n"/>
+      <c r="D57" s="20" t="n"/>
+      <c r="E57" s="20" t="n"/>
+      <c r="F57" s="20" t="n"/>
+      <c r="G57" s="20" t="n"/>
+      <c r="H57" s="20" t="n"/>
+      <c r="I57" s="20" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="A58" s="20" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B58" s="19" t="n"/>
-      <c r="C58" s="29" t="inlineStr">
+      <c r="B58" s="20" t="n"/>
+      <c r="C58" s="30" t="inlineStr">
         <is>
           <t>Gravas arcillosas, mezclas grava-arena-arcilla.</t>
         </is>
       </c>
-      <c r="D58" s="19" t="n"/>
-      <c r="E58" s="19" t="n"/>
-      <c r="F58" s="19" t="n"/>
-      <c r="G58" s="19" t="n"/>
-      <c r="H58" s="19" t="n"/>
-      <c r="I58" s="19" t="n"/>
+      <c r="D58" s="20" t="n"/>
+      <c r="E58" s="20" t="n"/>
+      <c r="F58" s="20" t="n"/>
+      <c r="G58" s="20" t="n"/>
+      <c r="H58" s="20" t="n"/>
+      <c r="I58" s="20" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="inlineStr">
+      <c r="A59" s="20" t="inlineStr">
         <is>
           <t>SW</t>
         </is>
       </c>
-      <c r="B59" s="19" t="n"/>
-      <c r="C59" s="29" t="inlineStr">
+      <c r="B59" s="20" t="n"/>
+      <c r="C59" s="30" t="inlineStr">
         <is>
           <t>Arenas bien graduadas, arenas con grava, pocos finos o sin finos.</t>
         </is>
       </c>
-      <c r="D59" s="19" t="n"/>
-      <c r="E59" s="19" t="n"/>
-      <c r="F59" s="19" t="n"/>
-      <c r="G59" s="19" t="n"/>
-      <c r="H59" s="19" t="n"/>
-      <c r="I59" s="19" t="n"/>
+      <c r="D59" s="20" t="n"/>
+      <c r="E59" s="20" t="n"/>
+      <c r="F59" s="20" t="n"/>
+      <c r="G59" s="20" t="n"/>
+      <c r="H59" s="20" t="n"/>
+      <c r="I59" s="20" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="inlineStr">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="B60" s="19" t="n"/>
-      <c r="C60" s="29" t="inlineStr">
+      <c r="B60" s="20" t="n"/>
+      <c r="C60" s="30" t="inlineStr">
         <is>
           <t>Arenas mal graduadas, arenas con grava, pocos finos o sin finos.</t>
         </is>
       </c>
-      <c r="D60" s="19" t="n"/>
-      <c r="E60" s="19" t="n"/>
-      <c r="F60" s="19" t="n"/>
-      <c r="G60" s="19" t="n"/>
-      <c r="H60" s="19" t="n"/>
-      <c r="I60" s="19" t="n"/>
+      <c r="D60" s="20" t="n"/>
+      <c r="E60" s="20" t="n"/>
+      <c r="F60" s="20" t="n"/>
+      <c r="G60" s="20" t="n"/>
+      <c r="H60" s="20" t="n"/>
+      <c r="I60" s="20" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="B61" s="19" t="n"/>
-      <c r="C61" s="29" t="inlineStr">
+      <c r="B61" s="20" t="n"/>
+      <c r="C61" s="30" t="inlineStr">
         <is>
           <t>Arenas limosas, mezclas de arena y limo.</t>
         </is>
       </c>
-      <c r="D61" s="19" t="n"/>
-      <c r="E61" s="19" t="n"/>
-      <c r="F61" s="19" t="n"/>
-      <c r="G61" s="19" t="n"/>
-      <c r="H61" s="19" t="n"/>
-      <c r="I61" s="19" t="n"/>
+      <c r="D61" s="20" t="n"/>
+      <c r="E61" s="20" t="n"/>
+      <c r="F61" s="20" t="n"/>
+      <c r="G61" s="20" t="n"/>
+      <c r="H61" s="20" t="n"/>
+      <c r="I61" s="20" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="19" t="inlineStr">
+      <c r="A62" s="20" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="B62" s="19" t="n"/>
-      <c r="C62" s="29" t="inlineStr">
+      <c r="B62" s="20" t="n"/>
+      <c r="C62" s="30" t="inlineStr">
         <is>
           <t>Arenas arcillosas, mezclas de arena y arcilla.</t>
         </is>
       </c>
-      <c r="D62" s="19" t="n"/>
-      <c r="E62" s="19" t="n"/>
-      <c r="F62" s="19" t="n"/>
-      <c r="G62" s="19" t="n"/>
-      <c r="H62" s="19" t="n"/>
-      <c r="I62" s="19" t="n"/>
+      <c r="D62" s="20" t="n"/>
+      <c r="E62" s="20" t="n"/>
+      <c r="F62" s="20" t="n"/>
+      <c r="G62" s="20" t="n"/>
+      <c r="H62" s="20" t="n"/>
+      <c r="I62" s="20" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="A63" s="20" t="inlineStr">
         <is>
           <t>ML</t>
         </is>
       </c>
-      <c r="B63" s="19" t="n"/>
-      <c r="C63" s="29" t="inlineStr">
+      <c r="B63" s="20" t="n"/>
+      <c r="C63" s="30" t="inlineStr">
         <is>
           <t>Limos inorgánicos y arenas muy finas, limos limpios, arenas finas, limosas o arcillosas.</t>
         </is>
       </c>
-      <c r="D63" s="19" t="n"/>
-      <c r="E63" s="19" t="n"/>
-      <c r="F63" s="19" t="n"/>
-      <c r="G63" s="19" t="n"/>
-      <c r="H63" s="19" t="n"/>
-      <c r="I63" s="19" t="n"/>
+      <c r="D63" s="20" t="n"/>
+      <c r="E63" s="20" t="n"/>
+      <c r="F63" s="20" t="n"/>
+      <c r="G63" s="20" t="n"/>
+      <c r="H63" s="20" t="n"/>
+      <c r="I63" s="20" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="19" t="inlineStr">
+      <c r="A64" s="20" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B64" s="19" t="n"/>
-      <c r="C64" s="29" t="inlineStr">
+      <c r="B64" s="20" t="n"/>
+      <c r="C64" s="30" t="inlineStr">
         <is>
           <t>Arcillas inorgánicas de plasticidad baja a media, arcillas con grava, arcillas arenosas.</t>
         </is>
       </c>
-      <c r="D64" s="19" t="n"/>
-      <c r="E64" s="19" t="n"/>
-      <c r="F64" s="19" t="n"/>
-      <c r="G64" s="19" t="n"/>
-      <c r="H64" s="19" t="n"/>
-      <c r="I64" s="19" t="n"/>
+      <c r="D64" s="20" t="n"/>
+      <c r="E64" s="20" t="n"/>
+      <c r="F64" s="20" t="n"/>
+      <c r="G64" s="20" t="n"/>
+      <c r="H64" s="20" t="n"/>
+      <c r="I64" s="20" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="19" t="inlineStr">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>OL</t>
         </is>
       </c>
-      <c r="B65" s="19" t="n"/>
-      <c r="C65" s="29" t="inlineStr">
+      <c r="B65" s="20" t="n"/>
+      <c r="C65" s="30" t="inlineStr">
         <is>
           <t>Limos orgánicos y arcillas orgánicas limosas de baja plasticidad.</t>
         </is>
       </c>
-      <c r="D65" s="19" t="n"/>
-      <c r="E65" s="19" t="n"/>
-      <c r="F65" s="19" t="n"/>
-      <c r="G65" s="19" t="n"/>
-      <c r="H65" s="19" t="n"/>
-      <c r="I65" s="19" t="n"/>
+      <c r="D65" s="20" t="n"/>
+      <c r="E65" s="20" t="n"/>
+      <c r="F65" s="20" t="n"/>
+      <c r="G65" s="20" t="n"/>
+      <c r="H65" s="20" t="n"/>
+      <c r="I65" s="20" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="19" t="inlineStr">
+      <c r="A66" s="20" t="inlineStr">
         <is>
           <t>MH</t>
         </is>
       </c>
-      <c r="B66" s="19" t="n"/>
-      <c r="C66" s="29" t="inlineStr">
+      <c r="B66" s="20" t="n"/>
+      <c r="C66" s="30" t="inlineStr">
         <is>
           <t>Limos inorgánicos, suelos arenosos finos o limosos con mica o diatomeas.</t>
         </is>
       </c>
-      <c r="D66" s="19" t="n"/>
-      <c r="E66" s="19" t="n"/>
-      <c r="F66" s="19" t="n"/>
-      <c r="G66" s="19" t="n"/>
-      <c r="H66" s="19" t="n"/>
-      <c r="I66" s="19" t="n"/>
+      <c r="D66" s="20" t="n"/>
+      <c r="E66" s="20" t="n"/>
+      <c r="F66" s="20" t="n"/>
+      <c r="G66" s="20" t="n"/>
+      <c r="H66" s="20" t="n"/>
+      <c r="I66" s="20" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="19" t="inlineStr">
+      <c r="A67" s="20" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="B67" s="19" t="n"/>
-      <c r="C67" s="29" t="inlineStr">
+      <c r="B67" s="20" t="n"/>
+      <c r="C67" s="30" t="inlineStr">
         <is>
           <t>Arcillas inorgánicas de plasticidad alta.</t>
         </is>
       </c>
-      <c r="D67" s="19" t="n"/>
-      <c r="E67" s="19" t="n"/>
-      <c r="F67" s="19" t="n"/>
-      <c r="G67" s="19" t="n"/>
-      <c r="H67" s="19" t="n"/>
-      <c r="I67" s="19" t="n"/>
+      <c r="D67" s="20" t="n"/>
+      <c r="E67" s="20" t="n"/>
+      <c r="F67" s="20" t="n"/>
+      <c r="G67" s="20" t="n"/>
+      <c r="H67" s="20" t="n"/>
+      <c r="I67" s="20" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="19" t="inlineStr">
+      <c r="A68" s="20" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="B68" s="19" t="n"/>
-      <c r="C68" s="29" t="inlineStr">
+      <c r="B68" s="20" t="n"/>
+      <c r="C68" s="30" t="inlineStr">
         <is>
           <t>Arcillas orgánicas de plasticidad media a alta.</t>
         </is>
       </c>
-      <c r="D68" s="19" t="n"/>
-      <c r="E68" s="19" t="n"/>
-      <c r="F68" s="19" t="n"/>
-      <c r="G68" s="19" t="n"/>
-      <c r="H68" s="19" t="n"/>
-      <c r="I68" s="19" t="n"/>
+      <c r="D68" s="20" t="n"/>
+      <c r="E68" s="20" t="n"/>
+      <c r="F68" s="20" t="n"/>
+      <c r="G68" s="20" t="n"/>
+      <c r="H68" s="20" t="n"/>
+      <c r="I68" s="20" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="16" t="inlineStr">
+      <c r="A70" s="17" t="inlineStr">
         <is>
           <t>CURVA GRANULOMÉTRICA</t>
         </is>
       </c>
-      <c r="B70" s="17" t="n"/>
-      <c r="C70" s="17" t="n"/>
-      <c r="D70" s="17" t="n"/>
-      <c r="E70" s="17" t="n"/>
-      <c r="F70" s="17" t="n"/>
-      <c r="G70" s="17" t="n"/>
-      <c r="H70" s="17" t="n"/>
-      <c r="I70" s="17" t="n"/>
+      <c r="B70" s="18" t="n"/>
+      <c r="C70" s="18" t="n"/>
+      <c r="D70" s="18" t="n"/>
+      <c r="E70" s="18" t="n"/>
+      <c r="F70" s="18" t="n"/>
+      <c r="G70" s="18" t="n"/>
+      <c r="H70" s="18" t="n"/>
+      <c r="I70" s="18" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="30" t="n"/>
-      <c r="B101" s="30" t="n"/>
-      <c r="C101" s="30" t="n"/>
-      <c r="D101" s="30" t="n"/>
-      <c r="E101" s="30" t="n"/>
-      <c r="F101" s="30" t="n"/>
-      <c r="G101" s="30" t="n"/>
-      <c r="H101" s="30" t="n"/>
-      <c r="I101" s="30" t="n"/>
+      <c r="A101" s="31" t="n"/>
+      <c r="B101" s="31" t="n"/>
+      <c r="C101" s="31" t="n"/>
+      <c r="D101" s="31" t="n"/>
+      <c r="E101" s="31" t="n"/>
+      <c r="F101" s="31" t="n"/>
+      <c r="G101" s="31" t="n"/>
+      <c r="H101" s="31" t="n"/>
+      <c r="I101" s="31" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="31" t="inlineStr">
+      <c r="A102" s="32" t="inlineStr">
         <is>
           <t>ESP. ENSAYOS GEOTECNICOS</t>
         </is>
       </c>
-      <c r="D102" s="31" t="inlineStr">
+      <c r="D102" s="32" t="inlineStr">
         <is>
           <t>ESP. SUELOS Y PAVIMENTOS</t>
         </is>
       </c>
-      <c r="G102" s="31" t="inlineStr">
+      <c r="G102" s="32" t="inlineStr">
         <is>
           <t>SUPERVISOR</t>
         </is>

</xml_diff>

<commit_message>
Tablas y bandas encuadradas en los informes Excel
- Proctor: DATOS DE ENSAYO y CÁLCULO DE LA HUMEDAD a ancho completo
  (M1-M4 distribuidas en pares de columnas hasta la columna I, como el
  PDF); cajas MDS/OCH a ancho completo
- Límites: bandas de sección al ancho exacto de su tabla (LL A:D,
  LP/HN A:C) y cajas de resultado alineadas a su tabla
- Granulometría: banda TAMIZADO al ancho de la tabla de tamices (A:F)
</commit_message>
<xml_diff>
--- a/backend/templates/base/base_granulometria.xlsx
+++ b/backend/templates/base/base_granulometria.xlsx
@@ -1184,9 +1184,6 @@
       <c r="D23" s="18" t="n"/>
       <c r="E23" s="18" t="n"/>
       <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
@@ -2247,7 +2244,7 @@
     <mergeCell ref="C1:G1"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A66:B66"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>

</xml_diff>

<commit_message>
Bordes completos en la ficha técnica de los informes Excel
par_ficha: los valores de una sola celda no recibían borde (el cuadro
quedaba abierto) y los estilos se aplicaban después de combinar, lo
que openpyxl no persiste; ahora estilos primero y merge después.
Proctor: el valor de Martillo (lb) se extiende hasta el borde derecho
para cerrar la fila COMPACTACIÓN.
</commit_message>
<xml_diff>
--- a/backend/templates/base/base_granulometria.xlsx
+++ b/backend/templates/base/base_granulometria.xlsx
@@ -264,15 +264,14 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -280,9 +279,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -996,14 +992,14 @@
       </c>
       <c r="B12" s="11" t="n"/>
       <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Fecha Muestreo:</t>
         </is>
       </c>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="16" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -1017,12 +1013,14 @@
         </is>
       </c>
       <c r="C13" s="10" t="n"/>
+      <c r="D13" s="13" t="n"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
           <t>N:</t>
         </is>
       </c>
       <c r="F13" s="10" t="n"/>
+      <c r="G13" s="13" t="n"/>
       <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Prof. (m):</t>
@@ -1041,25 +1039,25 @@
           <t>Explor.:</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n"/>
+      <c r="C14" s="11" t="n"/>
       <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Progresiva:</t>
         </is>
       </c>
-      <c r="E14" s="16" t="n"/>
+      <c r="E14" s="11" t="n"/>
       <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Estrato:</t>
         </is>
       </c>
-      <c r="G14" s="16" t="n"/>
+      <c r="G14" s="11" t="n"/>
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Lado:</t>
         </is>
       </c>
-      <c r="I14" s="16" t="n"/>
+      <c r="I14" s="11" t="n"/>
     </row>
     <row r="15" ht="6" customHeight="1"/>
     <row r="16">
@@ -1078,24 +1076,24 @@
       <c r="I16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>PESO TOTAL (g)</t>
         </is>
       </c>
       <c r="B17" s="19" t="n"/>
       <c r="C17" s="20" t="n"/>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>PESO FRAC. FINA TAMIZADA (g)</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n"/>
+      <c r="E17" s="15" t="n"/>
       <c r="F17" s="19" t="n"/>
       <c r="G17" s="20" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>PESO FRACCIÓN GRUESA (g)</t>
         </is>
@@ -1105,12 +1103,12 @@
         <v/>
       </c>
       <c r="C18" s="22" t="n"/>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>PESO MUESTRA LAVADA (g)</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n"/>
+      <c r="E18" s="15" t="n"/>
       <c r="F18" s="21">
         <f>IF(AND(N(B17)&gt;0,N(F17)&gt;0),B18+SUM(C35:C45)*B19/F17,"")</f>
         <v/>
@@ -1118,7 +1116,7 @@
       <c r="G18" s="22" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>PESO FRACCIÓN FINA (g)</t>
         </is>
@@ -1128,12 +1126,12 @@
         <v/>
       </c>
       <c r="C19" s="22" t="n"/>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>COEFICIENTE</t>
         </is>
       </c>
-      <c r="E19" s="14" t="n"/>
+      <c r="E19" s="15" t="n"/>
       <c r="F19" s="23">
         <f>IF(AND(N(B17)&gt;0,N(F17)&gt;0),IFERROR(F17/B17,0),"")</f>
         <v/>
@@ -1141,24 +1139,24 @@
       <c r="G19" s="22" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>LÍMITE LÍQUIDO (%)</t>
         </is>
       </c>
       <c r="B20" s="19" t="n"/>
       <c r="C20" s="20" t="n"/>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>ÍNDICE DE PLASTICIDAD (%)</t>
         </is>
       </c>
-      <c r="E20" s="14" t="n"/>
+      <c r="E20" s="15" t="n"/>
       <c r="F20" s="19" t="n"/>
       <c r="G20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>GRADACIÓN</t>
         </is>
@@ -1830,7 +1828,7 @@
       <c r="I49" s="18" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>% GRAVA</t>
         </is>
@@ -1839,7 +1837,7 @@
         <f>IF(ISNUMBER(E34),E34,"")</f>
         <v/>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>% ARENA</t>
         </is>
@@ -1849,7 +1847,7 @@
         <v/>
       </c>
       <c r="E50" s="9" t="n"/>
-      <c r="F50" s="13" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
         <is>
           <t>% FINOS</t>
         </is>
@@ -1862,7 +1860,7 @@
       <c r="I50" s="9" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>TMN</t>
         </is>

</xml_diff>